<commit_message>
[refactor]: new DER + sample data + SQL code
</commit_message>
<xml_diff>
--- a/data/dados-banco-api.xlsx
+++ b/data/dados-banco-api.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://embraer-my.sharepoint.com/personal/natan_telles_embraer_com_br/Documents/Documents/Público/FATEC/sistema-gerenciador-provas/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5E9918CC-FA26-48E3-9992-04E91D8ACA74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{5E9918CC-FA26-48E3-9992-04E91D8ACA74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CC41733-6D4A-4C6A-A168-F0DBD146F03D}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{6084E485-0BAD-48C1-A1BE-B06EC2C0E63D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{6084E485-0BAD-48C1-A1BE-B06EC2C0E63D}"/>
   </bookViews>
   <sheets>
     <sheet name="Prova" sheetId="1" r:id="rId1"/>
     <sheet name="Questao" sheetId="2" r:id="rId2"/>
-    <sheet name="Alternativa" sheetId="3" r:id="rId3"/>
+    <sheet name="Prova_Questao" sheetId="5" r:id="rId3"/>
+    <sheet name="Alternativa" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -55,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="74">
   <si>
     <t>codigo</t>
   </si>
@@ -153,9 +154,6 @@
     <t xml:space="preserve"> SQL                               </t>
   </si>
   <si>
-    <t xml:space="preserve"> AMD01        </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Qual a função de uma chave primária?                 </t>
   </si>
   <si>
@@ -165,27 +163,15 @@
     <t xml:space="preserve"> O que representa um relacionamento 1:N?              </t>
   </si>
   <si>
-    <t xml:space="preserve"> LDP01        </t>
-  </si>
-  <si>
     <t xml:space="preserve"> O que é um objeto em POO?                            </t>
   </si>
   <si>
-    <t xml:space="preserve"> POO01        </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Qual conceito permite reutilização de código?        </t>
   </si>
   <si>
-    <t xml:space="preserve"> SBD01        </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Qual comando é utilizado para consultar dados?       </t>
   </si>
   <si>
-    <t xml:space="preserve"> SQL01        </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Qual cláusula filtra registros em uma consulta SQL?  </t>
   </si>
   <si>
@@ -283,13 +269,22 @@
   </si>
   <si>
     <t xml:space="preserve"> c) Um tipo de banco NoSQL                              </t>
+  </si>
+  <si>
+    <t>POO01</t>
+  </si>
+  <si>
+    <t>SBD01</t>
+  </si>
+  <si>
+    <t>SQL01</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -319,16 +314,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -336,40 +350,257 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="11">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -394,7 +625,7 @@
     <tableColumn id="1" xr3:uid="{B9D57DB6-AA85-4340-A6AD-73C95C609923}" name="codigo"/>
     <tableColumn id="2" xr3:uid="{B40E20AB-43F7-4F38-8CE9-3EE373324326}" name="titulo"/>
     <tableColumn id="3" xr3:uid="{16D64877-2310-4BA2-9140-4BF38BEF8E31}" name="materia"/>
-    <tableColumn id="4" xr3:uid="{86313C83-82A3-449C-BA66-6AF8FDC9A3D9}" name="data_prova" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{86313C83-82A3-449C-BA66-6AF8FDC9A3D9}" name="data_prova" dataDxfId="7"/>
     <tableColumn id="5" xr3:uid="{0D77D392-AFB3-43E3-92A2-7FF970E86571}" name="curso"/>
     <tableColumn id="6" xr3:uid="{EADEAA82-9DE3-4A2B-89C3-F439D75E9A85}" name="bimestre"/>
   </tableColumns>
@@ -403,11 +634,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8CBD4544-95A2-46A5-870D-A161B857C399}" name="Questao" displayName="Questao" ref="A1:D11" totalsRowShown="0">
-  <autoFilter ref="A1:D11" xr:uid="{8CBD4544-95A2-46A5-870D-A161B857C399}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{BFE15401-EB7F-4270-AF6E-4C510F4906C5}" name="id_questao" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{4C9D6897-9195-4764-A469-6933FB125DA9}" name="codigo_prova"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8CBD4544-95A2-46A5-870D-A161B857C399}" name="Questao" displayName="Questao" ref="A1:C11" totalsRowShown="0">
+  <autoFilter ref="A1:C11" xr:uid="{8CBD4544-95A2-46A5-870D-A161B857C399}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{BFE15401-EB7F-4270-AF6E-4C510F4906C5}" name="id_questao" dataDxfId="6"/>
     <tableColumn id="3" xr3:uid="{67327181-A5C8-4884-B9CC-94EF1DC3D795}" name="titulo"/>
     <tableColumn id="4" xr3:uid="{5DE43BDD-4818-441E-A511-9F3CA6B69DEC}" name="descricao"/>
   </tableColumns>
@@ -416,12 +646,23 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{DFAB8622-420F-4E06-BBAE-412170F82CAA}" name="Tabela1" displayName="Tabela1" ref="A1:B11" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+  <autoFilter ref="A1:B11" xr:uid="{DFAB8622-420F-4E06-BBAE-412170F82CAA}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{9C06C47D-0E49-465B-8071-CA5A8BA21CE3}" name="codigo_prova" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{8ACA6414-A003-46C2-B0C3-4C0871355EBD}" name="id_questao" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F620FA8E-9AAC-481A-985F-877B1D3361F6}" name="Alternativa" displayName="Alternativa" ref="A1:D31" totalsRowShown="0">
   <autoFilter ref="A1:D31" xr:uid="{F620FA8E-9AAC-481A-985F-877B1D3361F6}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{6F7348DA-5339-492D-AF00-B36953075869}" name="id_alternativa" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{F843E4EB-8E8A-49C1-B580-0237C23DF2E0}" name="id_questao" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{7CB4BAE0-D66A-4CE8-91E4-BE09EDDA000A}" name="texto" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{6F7348DA-5339-492D-AF00-B36953075869}" name="id_alternativa" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{F843E4EB-8E8A-49C1-B580-0237C23DF2E0}" name="id_questao" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{7CB4BAE0-D66A-4CE8-91E4-BE09EDDA000A}" name="texto" dataDxfId="8"/>
     <tableColumn id="4" xr3:uid="{080F3D30-8CB8-4D19-ADF2-50CBC079DCD0}" name="correta"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -820,19 +1061,19 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="A5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" t="s">
         <v>24</v>
       </c>
       <c r="D5" s="2">
         <v>46305</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" t="s">
         <v>25</v>
       </c>
       <c r="F5">
@@ -840,19 +1081,19 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+      <c r="A6" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" t="s">
         <v>28</v>
       </c>
       <c r="D6" s="2">
         <v>46300</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" t="s">
         <v>25</v>
       </c>
       <c r="F6">
@@ -860,19 +1101,19 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+      <c r="A7" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" t="s">
         <v>31</v>
       </c>
       <c r="D7" s="2">
         <v>46310</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" t="s">
         <v>25</v>
       </c>
       <c r="F7">
@@ -880,16 +1121,16 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B9" s="5"/>
+      <c r="B9" s="4"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B10" s="5"/>
+      <c r="B10" s="4"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B11" s="5"/>
+      <c r="B11" s="4"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B12" s="5"/>
+      <c r="B12" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -901,174 +1142,135 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3385C8B4-B4AE-48BF-8AA8-ECF741D2C294}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.6328125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" customWidth="1"/>
-    <col min="3" max="3" width="26.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="B5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="6"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D12" s="7"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C14" s="7"/>
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -1079,8 +1281,116 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D031591-E05B-482A-828A-0C69E32E04F9}">
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.54296875" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43F78D12-383C-400B-A222-702AF7A346D7}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.7265625" style="3" customWidth="1"/>
@@ -1088,11 +1398,11 @@
     <col min="3" max="3" width="42.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" t="s">
         <v>13</v>
       </c>
       <c r="C1" t="s">
@@ -1102,215 +1412,217 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>46</v>
+      <c r="C2" t="s">
+        <v>41</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>47</v>
+      <c r="C3" t="s">
+        <v>42</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>48</v>
+      <c r="C4" t="s">
+        <v>43</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>49</v>
+      <c r="C5" t="s">
+        <v>44</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>50</v>
+      <c r="C6" t="s">
+        <v>45</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>51</v>
+      <c r="C7" t="s">
+        <v>46</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>52</v>
+      <c r="C8" t="s">
+        <v>47</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>53</v>
+      <c r="C9" t="s">
+        <v>48</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1</v>
       </c>
       <c r="B10">
         <v>9</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>54</v>
+      <c r="C10" t="s">
+        <v>49</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1</v>
       </c>
       <c r="B11">
         <v>10</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>55</v>
+      <c r="C11" t="s">
+        <v>50</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>56</v>
+      <c r="C12" t="s">
+        <v>51</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2</v>
       </c>
       <c r="B13">
         <v>2</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>57</v>
+      <c r="C13" t="s">
+        <v>52</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2</v>
       </c>
       <c r="B14">
         <v>3</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>58</v>
+      <c r="C14" s="5" t="s">
+        <v>53</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>2</v>
       </c>
       <c r="B15">
         <v>4</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>59</v>
+      <c r="C15" t="s">
+        <v>54</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>2</v>
       </c>
       <c r="B16">
         <v>5</v>
       </c>
-      <c r="C16" s="6" t="s">
-        <v>60</v>
+      <c r="C16" t="s">
+        <v>55</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
+      <c r="F16" s="5"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
@@ -1319,8 +1631,8 @@
       <c r="B17">
         <v>6</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>61</v>
+      <c r="C17" t="s">
+        <v>56</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -1333,8 +1645,8 @@
       <c r="B18">
         <v>7</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>62</v>
+      <c r="C18" t="s">
+        <v>57</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -1347,8 +1659,8 @@
       <c r="B19">
         <v>8</v>
       </c>
-      <c r="C19" s="6" t="s">
-        <v>63</v>
+      <c r="C19" t="s">
+        <v>58</v>
       </c>
       <c r="D19">
         <v>0</v>
@@ -1361,8 +1673,8 @@
       <c r="B20">
         <v>9</v>
       </c>
-      <c r="C20" s="6" t="s">
-        <v>64</v>
+      <c r="C20" t="s">
+        <v>59</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -1375,8 +1687,8 @@
       <c r="B21">
         <v>10</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>65</v>
+      <c r="C21" t="s">
+        <v>60</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -1389,8 +1701,8 @@
       <c r="B22">
         <v>1</v>
       </c>
-      <c r="C22" s="6" t="s">
-        <v>66</v>
+      <c r="C22" t="s">
+        <v>61</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -1403,8 +1715,8 @@
       <c r="B23">
         <v>2</v>
       </c>
-      <c r="C23" s="6" t="s">
-        <v>67</v>
+      <c r="C23" t="s">
+        <v>62</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -1417,8 +1729,8 @@
       <c r="B24">
         <v>3</v>
       </c>
-      <c r="C24" s="6" t="s">
-        <v>68</v>
+      <c r="C24" t="s">
+        <v>63</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -1431,8 +1743,8 @@
       <c r="B25">
         <v>4</v>
       </c>
-      <c r="C25" s="6" t="s">
-        <v>69</v>
+      <c r="C25" t="s">
+        <v>64</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -1445,8 +1757,8 @@
       <c r="B26">
         <v>5</v>
       </c>
-      <c r="C26" s="6" t="s">
-        <v>70</v>
+      <c r="C26" t="s">
+        <v>65</v>
       </c>
       <c r="D26">
         <v>0</v>
@@ -1459,8 +1771,8 @@
       <c r="B27">
         <v>6</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>71</v>
+      <c r="C27" t="s">
+        <v>66</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -1473,8 +1785,8 @@
       <c r="B28">
         <v>7</v>
       </c>
-      <c r="C28" s="6" t="s">
-        <v>72</v>
+      <c r="C28" t="s">
+        <v>67</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -1487,8 +1799,8 @@
       <c r="B29">
         <v>8</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>73</v>
+      <c r="C29" t="s">
+        <v>68</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1501,8 +1813,8 @@
       <c r="B30">
         <v>9</v>
       </c>
-      <c r="C30" s="6" t="s">
-        <v>74</v>
+      <c r="C30" t="s">
+        <v>69</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -1515,8 +1827,8 @@
       <c r="B31">
         <v>10</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>75</v>
+      <c r="C31" t="s">
+        <v>70</v>
       </c>
       <c r="D31">
         <v>0</v>

</xml_diff>